<commit_message>
Add program terrain, phase brackets and weekly schedule overlay
Weekly target-km bars per runner under the track, dated phase brackets
with km/long-run summary, hover detail, and a click-through overlay with
the Monday-Sunday schedule read from the Kalender sheet (actual km,
coaching notes, prev/next week, runner tabs, mobile bottom sheet).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F6YBYKzuMdPjhKBp8CabRD
</commit_message>
<xml_diff>
--- a/tests/fixtures/program_mini.xlsx
+++ b/tests/fixtures/program_mini.xlsx
@@ -562,13 +562,35 @@
           <t>1 Base</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>ISTIRAHAT PENUH</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Lari santai 5 km
+Detak jantung 139 - 152</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Lari santai 5 km</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>LONG RUN 14 km
+Perkiraan waktu: 2 jam</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Lari pemulihan 4 km</t>
+        </is>
+      </c>
       <c r="K4" t="n">
         <v>28</v>
       </c>
@@ -595,13 +617,35 @@
           <t>1 Base</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>ISTIRAHAT PENUH</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Lari santai 5 km
+Detak jantung 139 - 152</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Lari santai 5 km</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>LONG RUN 12 km
+Perkiraan waktu: 2 jam</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Lari pemulihan 4 km</t>
+        </is>
+      </c>
       <c r="K5" t="n">
         <v>24</v>
       </c>
@@ -628,13 +672,35 @@
           <t>2 Support</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ISTIRAHAT PENUH</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Lari santai 5 km
+Detak jantung 139 - 152</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Lari santai 5 km</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>LONG RUN - km
+Perkiraan waktu: 2 jam</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Lari pemulihan 4 km</t>
+        </is>
+      </c>
       <c r="K6" t="n">
         <v>21</v>
       </c>
@@ -663,13 +729,35 @@
           <t>2 Support</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>ISTIRAHAT PENUH</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Lari santai 5 km
+Detak jantung 139 - 152</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Lari santai 5 km</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>LONG RUN 20 km
+Perkiraan waktu: 2 jam</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Lari pemulihan 4 km</t>
+        </is>
+      </c>
       <c r="K7" t="n">
         <v>35</v>
       </c>

</xml_diff>